<commit_message>
Add game entry: 4545
</commit_message>
<xml_diff>
--- a/Gameday Plan.xlsx
+++ b/Gameday Plan.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -859,9 +859,32 @@
         <v>adsdas</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Boardgames</v>
+      </c>
+      <c r="B21" t="str">
+        <v>4545</v>
+      </c>
+      <c r="C21" t="str">
+        <v>4545</v>
+      </c>
+      <c r="D21" t="str">
+        <v>4545</v>
+      </c>
+      <c r="E21" t="str">
+        <v>4554</v>
+      </c>
+      <c r="F21" t="str">
+        <v>4545</v>
+      </c>
+      <c r="G21" t="str">
+        <v>4545</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>